<commit_message>
Agregar capturas responsive y actualizar matriz de trazabilidad
</commit_message>
<xml_diff>
--- a/docs/Matriz_Trazabilidad.xlsx
+++ b/docs/Matriz_Trazabilidad.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
   <si>
-    <t>Requisitos</t>
+    <t>Requerimientos</t>
   </si>
   <si>
     <t>Requisito</t>
@@ -22,7 +22,7 @@
     <t xml:space="preserve">Archivo </t>
   </si>
   <si>
-    <t>Requisito 1</t>
+    <t>RF-01</t>
   </si>
   <si>
     <t>Crear una página principal con información de QuestPass CR.</t>
@@ -31,7 +31,7 @@
     <t>index.html</t>
   </si>
   <si>
-    <t>Requisito 2</t>
+    <t>RF-02</t>
   </si>
   <si>
     <t>Mostrar un catálogo con seis experiencias.</t>
@@ -40,7 +40,7 @@
     <t>experiencias.html</t>
   </si>
   <si>
-    <t>Requisito 3</t>
+    <t>RF-03</t>
   </si>
   <si>
     <t>Mostrar los detalles de la experiencia QST-001.</t>
@@ -49,7 +49,7 @@
     <t>detalle.html</t>
   </si>
   <si>
-    <t>Requisito 4</t>
+    <t>RF-04</t>
   </si>
   <si>
     <t>Crear un formulario de reservas.</t>
@@ -58,13 +58,13 @@
     <t>reservar.html</t>
   </si>
   <si>
-    <t>Requisito 5</t>
+    <t>RF-05</t>
   </si>
   <si>
     <t>Validar los campos obligatorios del formulario de reservas.</t>
   </si>
   <si>
-    <t>Requisito 6</t>
+    <t>RF-06</t>
   </si>
   <si>
     <t>Crear un formulario de contacto.</t>
@@ -73,7 +73,7 @@
     <t>contacto.html</t>
   </si>
   <si>
-    <t>Requisito 7</t>
+    <t>RF-07</t>
   </si>
   <si>
     <t>Crear un formulario de inicio de sesión.</t>
@@ -82,7 +82,7 @@
     <t>login.html</t>
   </si>
   <si>
-    <t>Requisito 8</t>
+    <t>RF-08</t>
   </si>
   <si>
     <t>Mostrar las experiencias en el panel de administración.</t>
@@ -91,13 +91,13 @@
     <t>admin.html</t>
   </si>
   <si>
-    <t>Requisito 9</t>
+    <t>RF-09</t>
   </si>
   <si>
     <t>Mostrar una tabla de reservas vacía.</t>
   </si>
   <si>
-    <t>Requisito 10</t>
+    <t>RF-10</t>
   </si>
   <si>
     <t>Implementar navegación entre las siete páginas.</t>
@@ -106,13 +106,13 @@
     <t>Todos los archivos HTML</t>
   </si>
   <si>
-    <t>Requisito 11</t>
+    <t>RF-11</t>
   </si>
   <si>
     <t>Utilizar etiquetas HTML semánticas y un único &lt;h1&gt; por página.</t>
   </si>
   <si>
-    <t>Requisito 12</t>
+    <t>RF-12</t>
   </si>
   <si>
     <t>Aplicar estilos CSS personalizados.</t>
@@ -121,13 +121,13 @@
     <t>css/styles.css</t>
   </si>
   <si>
-    <t>Requisito 13</t>
+    <t>RF-13</t>
   </si>
   <si>
     <t>Implementar un diseño adaptable a dispositivos móviles y computadoras.</t>
   </si>
   <si>
-    <t>Requisito 14</t>
+    <t>RF-14</t>
   </si>
   <si>
     <t>Incorporar etiquetas visibles y estilos de foco para mejorar la accesibilidad.</t>

</xml_diff>